<commit_message>
commti - 7 "AI changes"
</commit_message>
<xml_diff>
--- a/qa-artifacts/FoodHub-Requirements-Checklist.xlsx
+++ b/qa-artifacts/FoodHub-Requirements-Checklist.xlsx
@@ -401,7 +401,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B7"/>
   <cols>
-    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -418,7 +418,7 @@
         <v>Covered</v>
       </c>
       <c r="B2">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3">
@@ -426,7 +426,7 @@
         <v>Mostly Covered</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -434,7 +434,7 @@
         <v>Partially Covered</v>
       </c>
       <c r="B4">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -442,7 +442,7 @@
         <v>Missing / Not Enforced</v>
       </c>
       <c r="B5">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -458,7 +458,7 @@
         <v>Not Covered</v>
       </c>
       <c r="B7">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -472,10 +472,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D62"/>
   <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
+    <col min="1" max="1" width="36.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="62.83203125" customWidth="1"/>
-    <col min="4" max="4" width="72.83203125" customWidth="1"/>
+    <col min="3" max="3" width="72.83203125" customWidth="1"/>
+    <col min="4" max="4" width="92.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -833,13 +833,13 @@
         <v>Unit test payment logic</v>
       </c>
       <c r="B26" t="str">
-        <v>Partially Covered</v>
+        <v>Covered</v>
       </c>
       <c r="C26" t="str">
-        <v>OrderService payment failure unit test</v>
+        <v>tests/unit/paymentService.test.ts and OrderService payment tests</v>
       </c>
       <c r="D26" t="str">
-        <v>Payment behavior is covered through service, but FakePaymentGateway token rules lack dedicated unit tests.</v>
+        <v>FakePaymentGateway token rules, non-positive amounts, declined tokens, non-gateway tokens, and approved payment IDs are directly unit tested.</v>
       </c>
     </row>
     <row r="27">
@@ -875,13 +875,13 @@
         <v>Critical logic 90%+ coverage</v>
       </c>
       <c r="B29" t="str">
-        <v>Missing / Not Enforced</v>
+        <v>Covered</v>
       </c>
       <c r="C29" t="str">
-        <v>No coverage script or threshold found</v>
+        <v>npm run test:coverage, vitest.config.ts thresholds, CI coverage-gate, qa-artifacts/coverage</v>
       </c>
       <c r="D29" t="str">
-        <v>A coverage gate would be needed to prove this.</v>
+        <v>Statements, branches, functions, and lines have 90% thresholds for critical service logic.</v>
       </c>
     </row>
     <row r="30">
@@ -1046,10 +1046,10 @@
         <v>Covered</v>
       </c>
       <c r="C41" t="str">
-        <v>.github/workflows PR Test Gate</v>
+        <v>.github/workflows/ci.yml pull_request trigger on main</v>
       </c>
       <c r="D41" t="str">
-        <v>Workflow triggers on pull requests to main.</v>
+        <v>Workflow triggers on opened, synchronize, reopened, and ready_for_review pull requests.</v>
       </c>
     </row>
     <row r="42">
@@ -1060,10 +1060,10 @@
         <v>Mostly Covered</v>
       </c>
       <c r="C42" t="str">
-        <v>Sequential command steps fail job on failures</v>
+        <v>.github/workflows/ci.yml independent jobs fail on command errors</v>
       </c>
       <c r="D42" t="str">
-        <v>Reports/artifacts still run with if: always after failures.</v>
+        <v>Test jobs fail on suite failures; QA artifact collection still runs with if: always to preserve diagnostics.</v>
       </c>
     </row>
     <row r="43">
@@ -1071,13 +1071,13 @@
         <v>CI parallel execution</v>
       </c>
       <c r="B43" t="str">
-        <v>Not Covered</v>
+        <v>Covered</v>
       </c>
       <c r="C43" t="str">
-        <v>Single workflow job runs suites sequentially</v>
+        <v>.github/workflows/ci.yml separate jobs for unit, integration, contract, coverage, E2E, and load tests</v>
       </c>
       <c r="D43" t="str">
-        <v>Would need separate jobs or matrix for true parallelism.</v>
+        <v>PR gate suites run as independent GitHub Actions jobs, with QA report generated after dependencies complete.</v>
       </c>
     </row>
     <row r="44">
@@ -1239,13 +1239,13 @@
         <v>Observability gap</v>
       </c>
       <c r="B55" t="str">
-        <v>Partially Covered</v>
+        <v>Mostly Covered</v>
       </c>
       <c r="C55" t="str">
-        <v>requestLogger exists</v>
+        <v>Structured request logs, observability JSON metrics, SQLite DB, Excel dashboard charts, QA Report Viewer refresh/open/truncate controls</v>
       </c>
       <c r="D55" t="str">
-        <v>Basic logs only; no metrics/tracing/alerts.</v>
+        <v>Local portable QA observability is implemented. Production-grade distributed tracing and external alerting remain out of scope.</v>
       </c>
     </row>
     <row r="56">
@@ -1355,12 +1355,12 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D8"/>
   <cols>
-    <col min="1" max="1" width="42.83203125" customWidth="1"/>
+    <col min="1" max="1" width="36.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="62.83203125" customWidth="1"/>
-    <col min="4" max="4" width="72.83203125" customWidth="1"/>
+    <col min="3" max="3" width="72.83203125" customWidth="1"/>
+    <col min="4" max="4" width="92.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1393,133 +1393,91 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Unit test payment logic</v>
+        <v>CI fail fast</v>
       </c>
       <c r="B3" t="str">
-        <v>Partially Covered</v>
+        <v>Mostly Covered</v>
       </c>
       <c r="C3" t="str">
-        <v>OrderService payment failure unit test</v>
+        <v>.github/workflows/ci.yml independent jobs fail on command errors</v>
       </c>
       <c r="D3" t="str">
-        <v>Payment behavior is covered through service, but FakePaymentGateway token rules lack dedicated unit tests.</v>
+        <v>Test jobs fail on suite failures; QA artifact collection still runs with if: always to preserve diagnostics.</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Critical logic 90%+ coverage</v>
+        <v>Observability gap</v>
       </c>
       <c r="B4" t="str">
-        <v>Missing / Not Enforced</v>
+        <v>Mostly Covered</v>
       </c>
       <c r="C4" t="str">
-        <v>No coverage script or threshold found</v>
+        <v>Structured logs, SQLite-backed metrics, Excel dashboard charts, viewer controls</v>
       </c>
       <c r="D4" t="str">
-        <v>A coverage gate would be needed to prove this.</v>
+        <v>Local QA observability is implemented; distributed tracing/external alerting are not part of this portable setup.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CI fail fast</v>
+        <v>AI-generated test suites add-on</v>
       </c>
       <c r="B5" t="str">
         <v>Mostly Covered</v>
       </c>
       <c r="C5" t="str">
-        <v>Sequential command steps fail job on failures</v>
+        <v>AI workbook/prompts and implemented suggested tests</v>
       </c>
       <c r="D5" t="str">
-        <v>Reports/artifacts still run with if: always after failures.</v>
+        <v>No live local model currently, by choice after performance concerns.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>CI parallel execution</v>
+        <v>Authentication SaaS risk</v>
       </c>
       <c r="B6" t="str">
-        <v>Not Covered</v>
+        <v>Missing / Known Gap</v>
       </c>
       <c r="C6" t="str">
-        <v>Single workflow job runs suites sequentially</v>
+        <v>No auth implementation found</v>
       </c>
       <c r="D6" t="str">
-        <v>Would need separate jobs or matrix for true parallelism.</v>
+        <v>Should be called out as future SaaS improvement.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Authentication SaaS risk</v>
+        <v>Rate limiting risk</v>
       </c>
       <c r="B7" t="str">
         <v>Missing / Known Gap</v>
       </c>
       <c r="C7" t="str">
-        <v>No auth implementation found</v>
+        <v>No rate limiting middleware found</v>
       </c>
       <c r="D7" t="str">
-        <v>Should be called out as future SaaS improvement.</v>
+        <v>Should be future enhancement.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Rate limiting risk</v>
+        <v>Payment idempotency risk</v>
       </c>
       <c r="B8" t="str">
         <v>Missing / Known Gap</v>
       </c>
       <c r="C8" t="str">
-        <v>No rate limiting middleware found</v>
+        <v>No idempotency key/duplicate payment prevention</v>
       </c>
       <c r="D8" t="str">
-        <v>Should be future enhancement.</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Payment idempotency risk</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Missing / Known Gap</v>
-      </c>
-      <c r="C9" t="str">
-        <v>No idempotency key/duplicate payment prevention</v>
-      </c>
-      <c r="D9" t="str">
         <v>Important future payment hardening item.</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Observability gap</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Partially Covered</v>
-      </c>
-      <c r="C10" t="str">
-        <v>requestLogger exists</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Basic logs only; no metrics/tracing/alerts.</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>AI-generated test suites add-on</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Mostly Covered</v>
-      </c>
-      <c r="C11" t="str">
-        <v>AI workbook/prompts and implemented suggested tests</v>
-      </c>
-      <c r="D11" t="str">
-        <v>No live local model currently, by choice after performance concerns.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>